<commit_message>
WordMaster 2000 Batch 6 and the final 2,000-word file
Batch 6 adds the last 262 words (126 from the HTML list, 91 written in
full, 45 from the 910-word workbook). The final file merges all batches,
drops the 69 removed words and renumbers 1-2,000.

Also fixes 13 Find & Fix lines that repeated their Common Mistake and
the Hindi meaning of right, well and please; moves shared row and
workbook code into sheet.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NoC3WZ9app4HCpgkAbzcVk
</commit_message>
<xml_diff>
--- a/content/wordmaster-2000/WordMaster2000_Batch5_Core_Words_1551-1807.xlsx
+++ b/content/wordmaster-2000/WordMaster2000_Batch5_Core_Words_1551-1807.xlsx
@@ -2469,7 +2469,7 @@
       </c>
       <c r="AX7" s="29" t="inlineStr">
         <is>
-          <t>We was late. → We were late.</t>
+          <t>They was at home. → They were at home.</t>
         </is>
       </c>
       <c r="AY7" s="29" t="inlineStr">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="AX11" s="29" t="inlineStr">
         <is>
-          <t>I can to swim. → I can swim.</t>
+          <t>She cans drive. → She can drive.</t>
         </is>
       </c>
       <c r="AY11" s="29" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="AX19" s="29" t="inlineStr">
         <is>
-          <t>How you are? → How are you?</t>
+          <t>How you know him? → How do you know him?</t>
         </is>
       </c>
       <c r="AY19" s="29" t="inlineStr">
@@ -12131,7 +12131,7 @@
       </c>
       <c r="AX42" s="29" t="inlineStr">
         <is>
-          <t>I weared a jacket. → I wore a jacket.</t>
+          <t>She is wearing glasses since childhood. → She has worn glasses since childhood.</t>
         </is>
       </c>
       <c r="AY42" s="29" t="inlineStr">
@@ -22204,7 +22204,7 @@
       </c>
       <c r="M79" s="29" t="inlineStr">
         <is>
-          <t>ठीक है ना? (पुष्टि के लिए)</t>
+          <t>सही / ठीक है ना?</t>
         </is>
       </c>
       <c r="N79" s="29" t="inlineStr">
@@ -28232,7 +28232,7 @@
       </c>
       <c r="M101" s="29" t="inlineStr">
         <is>
-          <t>अच्छा... (बातचीत शुरू करने के लिए)</t>
+          <t>अच्छी तरह / अच्छा… (बात शुरू करने के लिए)</t>
         </is>
       </c>
       <c r="N101" s="29" t="inlineStr">

</xml_diff>